<commit_message>
Harden NDI product media synchronization
</commit_message>
<xml_diff>
--- a/application/tests/Fixtures/Ndi/duplicate_sku.xlsx
+++ b/application/tests/Fixtures/Ndi/duplicate_sku.xlsx
@@ -542,7 +542,7 @@
       </x:c>
       <x:c r="AF2" s="10"/>
       <x:c r="AG2" s="10" t="str">
-        <x:v>https://example.invalid/TEST-TIRE-001.png</x:v>
+        <x:v>https://example.invalid/Imagev2.aspx?id=11111111-1111-4111-8111-111111111111</x:v>
       </x:c>
       <x:c r="AH2" s="10" t="str">
         <x:v>TEST-DOT25</x:v>
@@ -638,7 +638,7 @@
       </x:c>
       <x:c r="AF3" s="11"/>
       <x:c r="AG3" s="11" t="str">
-        <x:v>https://example.invalid/TEST-TIRE-001.png</x:v>
+        <x:v>https://example.invalid/Imagev2.aspx?id=11111111-1111-4111-8111-111111111111</x:v>
       </x:c>
       <x:c r="AH3" s="11" t="str">
         <x:v>TEST-DOT25</x:v>

</xml_diff>